<commit_message>
Change duration to story points in WBS
</commit_message>
<xml_diff>
--- a/Contx_WBS.xlsx
+++ b/Contx_WBS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mel\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user4\Downloads\CAPSTONE-THESIS\capdocs-panic\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E28EBD95-D935-47E6-BE59-C2279AC51363}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1463B7-63DF-4B3A-B67F-B124CDFFF3C6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WBS" sheetId="1" r:id="rId1"/>
@@ -35,9 +35,6 @@
     <t>Assigned Dev</t>
   </si>
   <si>
-    <t>Duration (days)</t>
-  </si>
-  <si>
     <t>Predecessor(s)</t>
   </si>
   <si>
@@ -876,6 +873,10 @@
   </si>
   <si>
     <t>- This is a teaching example; adjust Dev count, durations, and start date to fit your own class project.</t>
+  </si>
+  <si>
+    <t>Story Points
+(1 = 1 hour)</t>
   </si>
 </sst>
 </file>
@@ -1459,18 +1460,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K88"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
-    <col min="2" max="2" width="45.88671875" style="45" customWidth="1"/>
+    <col min="2" max="2" width="45.85546875" style="45" customWidth="1"/>
     <col min="3" max="3" width="46" style="45" customWidth="1"/>
     <col min="4" max="5" width="14" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
     <col min="7" max="10" width="16" customWidth="1"/>
-    <col min="11" max="11" width="15.6640625" style="53" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.7109375" style="53" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1484,66 +1485,66 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="20" t="s">
+      <c r="B2" s="21" t="s">
         <v>11</v>
-      </c>
-      <c r="B2" s="21" t="s">
-        <v>12</v>
       </c>
       <c r="C2" s="21"/>
       <c r="D2" s="20"/>
       <c r="E2" s="22"/>
       <c r="F2" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G2" s="23"/>
       <c r="H2" s="23"/>
       <c r="I2" s="24"/>
       <c r="J2" s="24"/>
       <c r="K2" s="46" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="29" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="3" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="29" t="s">
+      <c r="B3" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="B3" s="30" t="s">
+      <c r="C3" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="26" t="s">
+      <c r="D3" s="25" t="s">
         <v>17</v>
-      </c>
-      <c r="D3" s="25" t="s">
-        <v>18</v>
       </c>
       <c r="E3" s="27">
         <v>1</v>
       </c>
       <c r="F3" s="25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G3" s="28">
         <v>46191</v>
@@ -1558,27 +1559,27 @@
         <v>46197</v>
       </c>
       <c r="K3" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="29" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="30" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="30" t="s">
+      <c r="C4" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="26" t="s">
-        <v>21</v>
-      </c>
       <c r="D4" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E4" s="27">
         <v>1</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G4" s="28">
         <v>46192</v>
@@ -1593,27 +1594,27 @@
         <v>46198</v>
       </c>
       <c r="K4" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="29" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="30" t="s">
+      <c r="C5" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="26" t="s">
-        <v>24</v>
-      </c>
       <c r="D5" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E5" s="27">
         <v>4</v>
       </c>
       <c r="F5" s="25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G5" s="28">
         <v>46193</v>
@@ -1628,48 +1629,48 @@
         <v>46202</v>
       </c>
       <c r="K5" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="21" t="s">
         <v>25</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>26</v>
       </c>
       <c r="C6" s="21"/>
       <c r="D6" s="20"/>
       <c r="E6" s="22"/>
       <c r="F6" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G6" s="23"/>
       <c r="H6" s="23"/>
       <c r="I6" s="24"/>
       <c r="J6" s="24"/>
       <c r="K6" s="48" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="25" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="7" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="25" t="s">
+      <c r="B7" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="C7" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="26" t="s">
+      <c r="D7" s="25" t="s">
         <v>30</v>
-      </c>
-      <c r="D7" s="25" t="s">
-        <v>31</v>
       </c>
       <c r="E7" s="27">
         <v>2</v>
       </c>
       <c r="F7" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G7" s="28">
         <v>46202</v>
@@ -1684,27 +1685,27 @@
         <v>46207</v>
       </c>
       <c r="K7" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
+        <v>31</v>
+      </c>
+      <c r="B8" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="C8" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="11" t="s">
-        <v>34</v>
-      </c>
       <c r="D8" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E8" s="12">
         <v>1</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G8" s="32">
         <v>46203</v>
@@ -1719,27 +1720,27 @@
         <v>46207</v>
       </c>
       <c r="K8" s="49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
+        <v>34</v>
+      </c>
+      <c r="B9" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="C9" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="11" t="s">
-        <v>37</v>
-      </c>
       <c r="D9" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E9" s="12">
         <v>1</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G9" s="32">
         <v>46203</v>
@@ -1754,27 +1755,27 @@
         <v>46207</v>
       </c>
       <c r="K9" s="49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="C10" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="11" t="s">
-        <v>40</v>
-      </c>
       <c r="D10" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E10" s="12">
         <v>1</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G10" s="32">
         <v>46203</v>
@@ -1789,27 +1790,27 @@
         <v>46207</v>
       </c>
       <c r="K10" s="49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="B11" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="C11" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="11" t="s">
-        <v>43</v>
-      </c>
       <c r="D11" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E11" s="12">
         <v>1</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G11" s="32">
         <v>46203</v>
@@ -1824,27 +1825,27 @@
         <v>46207</v>
       </c>
       <c r="K11" s="49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
+        <v>43</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="C12" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="11" t="s">
-        <v>46</v>
-      </c>
       <c r="D12" s="10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E12" s="12">
         <v>1</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G12" s="32">
         <v>46203</v>
@@ -1859,27 +1860,27 @@
         <v>46207</v>
       </c>
       <c r="K12" s="49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="25" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="26" t="s">
+      <c r="C13" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="26" t="s">
-        <v>49</v>
-      </c>
       <c r="D13" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E13" s="27">
         <v>2</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G13" s="28">
         <v>46202</v>
@@ -1894,27 +1895,27 @@
         <v>46207</v>
       </c>
       <c r="K13" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="25" t="s">
+        <v>49</v>
+      </c>
+      <c r="B14" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="B14" s="26" t="s">
+      <c r="C14" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="C14" s="26" t="s">
+      <c r="D14" s="26" t="s">
         <v>52</v>
-      </c>
-      <c r="D14" s="26" t="s">
-        <v>53</v>
       </c>
       <c r="E14" s="27">
         <v>2</v>
       </c>
       <c r="F14" s="25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G14" s="28">
         <v>46233</v>
@@ -1925,27 +1926,27 @@
       <c r="I14" s="31"/>
       <c r="J14" s="31"/>
       <c r="K14" s="49" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="25" t="s">
         <v>54</v>
       </c>
-    </row>
-    <row r="15" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="25" t="s">
+      <c r="B15" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="26" t="s">
+      <c r="C15" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="C15" s="26" t="s">
-        <v>57</v>
-      </c>
       <c r="D15" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15" s="27">
         <v>2</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G15" s="28">
         <v>46237</v>
@@ -1956,27 +1957,27 @@
       <c r="I15" s="31"/>
       <c r="J15" s="31"/>
       <c r="K15" s="49" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="B16" s="26" t="s">
+      <c r="C16" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="C16" s="26" t="s">
+      <c r="D16" s="25" t="s">
         <v>60</v>
-      </c>
-      <c r="D16" s="25" t="s">
-        <v>61</v>
       </c>
       <c r="E16" s="27">
         <v>1</v>
       </c>
       <c r="F16" s="25" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G16" s="28">
         <v>46239</v>
@@ -1987,27 +1988,27 @@
       <c r="I16" s="31"/>
       <c r="J16" s="31"/>
       <c r="K16" s="49" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="25" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B17" s="26" t="s">
+      <c r="C17" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="C17" s="26" t="s">
-        <v>64</v>
-      </c>
       <c r="D17" s="25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E17" s="27">
         <v>2</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G17" s="28">
         <v>46202</v>
@@ -2022,48 +2023,48 @@
         <v>46207</v>
       </c>
       <c r="K17" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" s="21" t="s">
         <v>65</v>
-      </c>
-      <c r="B18" s="21" t="s">
-        <v>66</v>
       </c>
       <c r="C18" s="21"/>
       <c r="D18" s="20"/>
       <c r="E18" s="22"/>
       <c r="F18" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G18" s="23"/>
       <c r="H18" s="23"/>
       <c r="I18" s="24"/>
       <c r="J18" s="24"/>
       <c r="K18" s="48" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="25" t="s">
+        <v>66</v>
+      </c>
+      <c r="B19" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="B19" s="26" t="s">
+      <c r="C19" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="C19" s="26" t="s">
-        <v>69</v>
-      </c>
       <c r="D19" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E19" s="27">
         <v>2</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G19" s="28">
         <v>46202</v>
@@ -2078,27 +2079,27 @@
         <v>46207</v>
       </c>
       <c r="K19" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="25" t="s">
+        <v>69</v>
+      </c>
+      <c r="B20" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="C20" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="C20" s="26" t="s">
-        <v>72</v>
-      </c>
       <c r="D20" s="33" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E20" s="27">
         <v>1</v>
       </c>
       <c r="F20" s="25" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G20" s="28">
         <v>46203</v>
@@ -2111,27 +2112,27 @@
       </c>
       <c r="J20" s="31"/>
       <c r="K20" s="49" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="25" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="25" t="s">
+      <c r="B21" s="26" t="s">
         <v>74</v>
       </c>
-      <c r="B21" s="26" t="s">
+      <c r="C21" s="26" t="s">
         <v>75</v>
       </c>
-      <c r="C21" s="26" t="s">
-        <v>76</v>
-      </c>
       <c r="D21" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E21" s="27">
         <v>1</v>
       </c>
       <c r="F21" s="25" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G21" s="28">
         <v>46203</v>
@@ -2144,27 +2145,27 @@
       </c>
       <c r="J21" s="31"/>
       <c r="K21" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B22" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="B22" s="26" t="s">
+      <c r="C22" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="C22" s="26" t="s">
-        <v>79</v>
-      </c>
       <c r="D22" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E22" s="27">
         <v>1</v>
       </c>
       <c r="F22" s="25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G22" s="28">
         <v>46203</v>
@@ -2177,27 +2178,27 @@
       </c>
       <c r="J22" s="31"/>
       <c r="K22" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" s="26" t="s">
         <v>80</v>
       </c>
-      <c r="B23" s="26" t="s">
+      <c r="C23" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="C23" s="26" t="s">
-        <v>82</v>
-      </c>
       <c r="D23" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E23" s="27">
         <v>1</v>
       </c>
       <c r="F23" s="25" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G23" s="28">
         <v>46203</v>
@@ -2210,48 +2211,48 @@
       </c>
       <c r="J23" s="31"/>
       <c r="K23" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B24" s="21" t="s">
         <v>83</v>
-      </c>
-      <c r="B24" s="21" t="s">
-        <v>84</v>
       </c>
       <c r="C24" s="21"/>
       <c r="D24" s="20"/>
       <c r="E24" s="22"/>
       <c r="F24" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G24" s="23"/>
       <c r="H24" s="23"/>
       <c r="I24" s="24"/>
       <c r="J24" s="24"/>
       <c r="K24" s="46" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="25" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="26" t="s">
+      <c r="C25" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="26" t="s">
-        <v>87</v>
-      </c>
       <c r="D25" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E25" s="27">
         <v>2</v>
       </c>
       <c r="F25" s="25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G25" s="28">
         <v>46202</v>
@@ -2266,27 +2267,27 @@
         <v>46207</v>
       </c>
       <c r="K25" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="B26" s="26" t="s">
+      <c r="C26" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="26" t="s">
-        <v>90</v>
-      </c>
       <c r="D26" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E26" s="27">
         <v>2</v>
       </c>
       <c r="F26" s="25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="G26" s="28">
         <v>46202</v>
@@ -2301,48 +2302,48 @@
         <v>46207</v>
       </c>
       <c r="K26" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="B27" s="21" t="s">
         <v>91</v>
-      </c>
-      <c r="B27" s="21" t="s">
-        <v>92</v>
       </c>
       <c r="C27" s="21"/>
       <c r="D27" s="20"/>
       <c r="E27" s="22"/>
       <c r="F27" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G27" s="23"/>
       <c r="H27" s="23"/>
       <c r="I27" s="24"/>
       <c r="J27" s="24"/>
       <c r="K27" s="46" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="25" t="s">
+        <v>92</v>
+      </c>
+      <c r="B28" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="B28" s="26" t="s">
+      <c r="C28" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="C28" s="26" t="s">
-        <v>95</v>
-      </c>
       <c r="D28" s="33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E28" s="27">
         <v>1</v>
       </c>
       <c r="F28" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G28" s="34">
         <v>46204</v>
@@ -2357,27 +2358,27 @@
         <v>46209</v>
       </c>
       <c r="K28" s="49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="25" t="s">
+        <v>95</v>
+      </c>
+      <c r="B29" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="B29" s="26" t="s">
+      <c r="C29" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="C29" s="26" t="s">
+      <c r="D29" s="25" t="s">
         <v>98</v>
-      </c>
-      <c r="D29" s="25" t="s">
-        <v>99</v>
       </c>
       <c r="E29" s="27">
         <v>1</v>
       </c>
       <c r="F29" s="25" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="G29" s="34">
         <v>46205</v>
@@ -2392,27 +2393,27 @@
         <v>46212</v>
       </c>
       <c r="K29" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="25" t="s">
+        <v>99</v>
+      </c>
+      <c r="B30" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="B30" s="26" t="s">
+      <c r="C30" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="C30" s="26" t="s">
-        <v>102</v>
-      </c>
       <c r="D30" s="25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E30" s="27">
         <v>1</v>
       </c>
       <c r="F30" s="25" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="G30" s="34">
         <v>46205</v>
@@ -2427,27 +2428,27 @@
         <v>46212</v>
       </c>
       <c r="K30" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A31" s="25" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="B31" s="26" t="s">
+      <c r="C31" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="C31" s="26" t="s">
-        <v>105</v>
-      </c>
       <c r="D31" s="33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E31" s="27">
         <v>1</v>
       </c>
       <c r="F31" s="25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G31" s="34">
         <v>46204</v>
@@ -2462,48 +2463,48 @@
         <v>46209</v>
       </c>
       <c r="K31" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="B32" s="21" t="s">
         <v>106</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>107</v>
       </c>
       <c r="C32" s="21"/>
       <c r="D32" s="20"/>
       <c r="E32" s="22"/>
       <c r="F32" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G32" s="23"/>
       <c r="H32" s="23"/>
       <c r="I32" s="24"/>
       <c r="J32" s="24"/>
       <c r="K32" s="48" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="B33" s="26" t="s">
+      <c r="C33" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="C33" s="26" t="s">
-        <v>110</v>
-      </c>
       <c r="D33" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E33" s="27">
         <v>2</v>
       </c>
       <c r="F33" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G33" s="34">
         <v>46208</v>
@@ -2518,27 +2519,27 @@
         <v>46213</v>
       </c>
       <c r="K33" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="B34" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="B34" s="26" t="s">
+      <c r="C34" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="C34" s="26" t="s">
-        <v>113</v>
-      </c>
       <c r="D34" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E34" s="27">
         <v>1</v>
       </c>
       <c r="F34" s="25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G34" s="28">
         <v>46210</v>
@@ -2553,27 +2554,27 @@
         <v>46214</v>
       </c>
       <c r="K34" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="25" t="s">
+        <v>113</v>
+      </c>
+      <c r="B35" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="B35" s="26" t="s">
+      <c r="C35" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="C35" s="26" t="s">
-        <v>116</v>
-      </c>
       <c r="D35" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E35" s="27">
         <v>3</v>
       </c>
       <c r="F35" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G35" s="28">
         <v>46235</v>
@@ -2584,48 +2585,48 @@
       <c r="I35" s="31"/>
       <c r="J35" s="31"/>
       <c r="K35" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
+        <v>116</v>
+      </c>
+      <c r="B36" s="21" t="s">
         <v>117</v>
-      </c>
-      <c r="B36" s="21" t="s">
-        <v>118</v>
       </c>
       <c r="C36" s="21"/>
       <c r="D36" s="20"/>
       <c r="E36" s="22"/>
       <c r="F36" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G36" s="23"/>
       <c r="H36" s="23"/>
       <c r="I36" s="24"/>
       <c r="J36" s="24"/>
       <c r="K36" s="46" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" s="25" t="s">
+        <v>118</v>
+      </c>
+      <c r="B37" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="C37" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="C37" s="26" t="s">
-        <v>121</v>
-      </c>
       <c r="D37" s="33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E37" s="27">
         <v>1</v>
       </c>
       <c r="F37" s="25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G37" s="28">
         <v>46197</v>
@@ -2640,27 +2641,27 @@
         <v>46205</v>
       </c>
       <c r="K37" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="25" t="s">
+        <v>121</v>
+      </c>
+      <c r="B38" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="B38" s="26" t="s">
+      <c r="C38" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="C38" s="26" t="s">
-        <v>124</v>
-      </c>
       <c r="D38" s="26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E38" s="27">
         <v>10</v>
       </c>
       <c r="F38" s="25" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="G38" s="28">
         <v>46197</v>
@@ -2675,27 +2676,27 @@
         <v>46214</v>
       </c>
       <c r="K38" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="B39" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="B39" s="26" t="s">
+      <c r="C39" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="C39" s="26" t="s">
-        <v>127</v>
-      </c>
       <c r="D39" s="26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E39" s="27">
         <v>10</v>
       </c>
       <c r="F39" s="25" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="G39" s="28">
         <v>46197</v>
@@ -2710,48 +2711,48 @@
         <v>46214</v>
       </c>
       <c r="K39" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A40" s="20" t="s">
+        <v>127</v>
+      </c>
+      <c r="B40" s="21" t="s">
         <v>128</v>
-      </c>
-      <c r="B40" s="21" t="s">
-        <v>129</v>
       </c>
       <c r="C40" s="21"/>
       <c r="D40" s="20"/>
       <c r="E40" s="22"/>
       <c r="F40" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G40" s="23"/>
       <c r="H40" s="23"/>
       <c r="I40" s="24"/>
       <c r="J40" s="24"/>
       <c r="K40" s="48" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B41" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="B41" s="26" t="s">
+      <c r="C41" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="C41" s="26" t="s">
-        <v>132</v>
-      </c>
       <c r="D41" s="33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E41" s="27">
         <v>1</v>
       </c>
       <c r="F41" s="25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G41" s="28">
         <v>46197</v>
@@ -2766,27 +2767,27 @@
         <v>46205</v>
       </c>
       <c r="K41" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" s="25" t="s">
+        <v>132</v>
+      </c>
+      <c r="B42" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="B42" s="26" t="s">
+      <c r="C42" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="C42" s="26" t="s">
-        <v>135</v>
-      </c>
       <c r="D42" s="25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E42" s="27">
         <v>3</v>
       </c>
       <c r="F42" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G42" s="28">
         <v>46233</v>
@@ -2797,27 +2798,27 @@
       <c r="I42" s="31"/>
       <c r="J42" s="31"/>
       <c r="K42" s="49" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="25" t="s">
+        <v>135</v>
+      </c>
+      <c r="B43" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="B43" s="26" t="s">
+      <c r="C43" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="C43" s="26" t="s">
-        <v>138</v>
-      </c>
       <c r="D43" s="33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E43" s="27">
         <v>2</v>
       </c>
       <c r="F43" s="25" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G43" s="28">
         <v>46233</v>
@@ -2828,27 +2829,27 @@
       <c r="I43" s="31"/>
       <c r="J43" s="31"/>
       <c r="K43" s="49" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="25" t="s">
+        <v>138</v>
+      </c>
+      <c r="B44" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="B44" s="26" t="s">
+      <c r="C44" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="C44" s="26" t="s">
-        <v>141</v>
-      </c>
       <c r="D44" s="25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E44" s="27">
         <v>1</v>
       </c>
       <c r="F44" s="25" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G44" s="34">
         <v>46208</v>
@@ -2863,48 +2864,48 @@
         <v>46213</v>
       </c>
       <c r="K44" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="20" t="s">
+        <v>141</v>
+      </c>
+      <c r="B45" s="21" t="s">
         <v>142</v>
-      </c>
-      <c r="B45" s="21" t="s">
-        <v>143</v>
       </c>
       <c r="C45" s="21"/>
       <c r="D45" s="20"/>
       <c r="E45" s="22"/>
       <c r="F45" s="20" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G45" s="23"/>
       <c r="H45" s="23"/>
       <c r="I45" s="24"/>
       <c r="J45" s="24"/>
       <c r="K45" s="48" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" s="25" t="s">
+        <v>143</v>
+      </c>
+      <c r="B46" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="B46" s="26" t="s">
+      <c r="C46" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="C46" s="26" t="s">
-        <v>146</v>
-      </c>
       <c r="D46" s="25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E46" s="27">
         <v>3</v>
       </c>
       <c r="F46" s="25" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G46" s="28">
         <v>46213</v>
@@ -2919,21 +2920,21 @@
         <v>46207</v>
       </c>
       <c r="K46" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A47" s="25" t="s">
+        <v>146</v>
+      </c>
+      <c r="B47" s="26" t="s">
         <v>147</v>
-      </c>
-      <c r="B47" s="26" t="s">
-        <v>148</v>
       </c>
       <c r="C47" s="26"/>
       <c r="D47" s="25"/>
       <c r="E47" s="27"/>
       <c r="F47" s="25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G47" s="28">
         <v>46216</v>
@@ -2944,27 +2945,27 @@
       <c r="I47" s="31"/>
       <c r="J47" s="31"/>
       <c r="K47" s="48" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B48" s="11" t="s">
         <v>149</v>
       </c>
-      <c r="B48" s="11" t="s">
+      <c r="C48" s="11" t="s">
         <v>150</v>
       </c>
-      <c r="C48" s="11" t="s">
-        <v>151</v>
-      </c>
       <c r="D48" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E48" s="12">
         <v>2</v>
       </c>
       <c r="F48" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G48" s="18">
         <v>46216</v>
@@ -2979,27 +2980,27 @@
         <v>46207</v>
       </c>
       <c r="K48" s="49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B49" s="11" t="s">
         <v>152</v>
       </c>
-      <c r="B49" s="11" t="s">
+      <c r="C49" s="11" t="s">
         <v>153</v>
       </c>
-      <c r="C49" s="11" t="s">
-        <v>154</v>
-      </c>
       <c r="D49" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E49" s="12">
         <v>1</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G49" s="18">
         <v>46220</v>
@@ -3014,21 +3015,21 @@
         <v>46207</v>
       </c>
       <c r="K49" s="49" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" s="25" t="s">
+        <v>154</v>
+      </c>
+      <c r="B50" s="26" t="s">
         <v>155</v>
-      </c>
-      <c r="B50" s="26" t="s">
-        <v>156</v>
       </c>
       <c r="C50" s="26"/>
       <c r="D50" s="25"/>
       <c r="E50" s="27"/>
       <c r="F50" s="25" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G50" s="28">
         <v>46221</v>
@@ -3041,25 +3042,25 @@
       </c>
       <c r="J50" s="31"/>
       <c r="K50" s="48" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B51" s="11" t="s">
         <v>157</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="C51" s="11" t="s">
         <v>158</v>
-      </c>
-      <c r="C51" s="11" t="s">
-        <v>159</v>
       </c>
       <c r="D51" s="10"/>
       <c r="E51" s="12">
         <v>2</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G51" s="18">
         <v>46221</v>
@@ -3072,25 +3073,25 @@
       </c>
       <c r="J51" s="13"/>
       <c r="K51" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="B52" s="11" t="s">
         <v>160</v>
       </c>
-      <c r="B52" s="11" t="s">
+      <c r="C52" s="11" t="s">
         <v>161</v>
-      </c>
-      <c r="C52" s="11" t="s">
-        <v>162</v>
       </c>
       <c r="D52" s="10"/>
       <c r="E52" s="12">
         <v>1</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G52" s="18">
         <v>46223</v>
@@ -3103,25 +3104,25 @@
       </c>
       <c r="J52" s="13"/>
       <c r="K52" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="10" t="s">
+        <v>162</v>
+      </c>
+      <c r="B53" s="11" t="s">
         <v>163</v>
       </c>
-      <c r="B53" s="11" t="s">
+      <c r="C53" s="11" t="s">
         <v>164</v>
-      </c>
-      <c r="C53" s="11" t="s">
-        <v>165</v>
       </c>
       <c r="D53" s="10"/>
       <c r="E53" s="12">
         <v>1</v>
       </c>
       <c r="F53" s="10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G53" s="18">
         <v>46224</v>
@@ -3134,25 +3135,25 @@
       </c>
       <c r="J53" s="13"/>
       <c r="K53" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" ht="26.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="10" t="s">
+        <v>165</v>
+      </c>
+      <c r="B54" s="11" t="s">
         <v>166</v>
       </c>
-      <c r="B54" s="11" t="s">
+      <c r="C54" s="11" t="s">
         <v>167</v>
-      </c>
-      <c r="C54" s="11" t="s">
-        <v>168</v>
       </c>
       <c r="D54" s="10"/>
       <c r="E54" s="12">
         <v>1</v>
       </c>
       <c r="F54" s="10" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G54" s="18">
         <v>46227</v>
@@ -3165,25 +3166,25 @@
       </c>
       <c r="J54" s="13"/>
       <c r="K54" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="B55" s="11" t="s">
         <v>169</v>
       </c>
-      <c r="B55" s="11" t="s">
+      <c r="C55" s="11" t="s">
         <v>170</v>
-      </c>
-      <c r="C55" s="11" t="s">
-        <v>171</v>
       </c>
       <c r="D55" s="10"/>
       <c r="E55" s="12">
         <v>1</v>
       </c>
       <c r="F55" s="10" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="G55" s="18">
         <v>46228</v>
@@ -3196,25 +3197,25 @@
       </c>
       <c r="J55" s="13"/>
       <c r="K55" s="49" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" s="25" t="s">
+        <v>171</v>
+      </c>
+      <c r="B56" s="26" t="s">
         <v>172</v>
       </c>
-      <c r="B56" s="26" t="s">
+      <c r="C56" s="26" t="s">
         <v>173</v>
-      </c>
-      <c r="C56" s="26" t="s">
-        <v>174</v>
       </c>
       <c r="D56" s="25"/>
       <c r="E56" s="27">
         <v>2</v>
       </c>
       <c r="F56" s="25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G56" s="28">
         <v>46229</v>
@@ -3225,27 +3226,27 @@
       <c r="I56" s="31"/>
       <c r="J56" s="31"/>
       <c r="K56" s="48" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" ht="27.6" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A57" s="25" t="s">
+        <v>174</v>
+      </c>
+      <c r="B57" s="26" t="s">
         <v>175</v>
       </c>
-      <c r="B57" s="26" t="s">
+      <c r="C57" s="26" t="s">
         <v>176</v>
       </c>
-      <c r="C57" s="26" t="s">
-        <v>177</v>
-      </c>
       <c r="D57" s="25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E57" s="27">
         <v>1</v>
       </c>
       <c r="F57" s="25" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G57" s="28">
         <v>46231</v>
@@ -3256,27 +3257,27 @@
       <c r="I57" s="31"/>
       <c r="J57" s="31"/>
       <c r="K57" s="48" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="B58" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="B58" s="15" t="s">
+      <c r="C58" s="15" t="s">
         <v>179</v>
       </c>
-      <c r="C58" s="15" t="s">
-        <v>180</v>
-      </c>
       <c r="D58" s="14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E58" s="16">
         <v>0</v>
       </c>
       <c r="F58" s="14" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G58" s="19">
         <v>46191</v>
@@ -3287,21 +3288,21 @@
       <c r="I58" s="17"/>
       <c r="J58" s="17"/>
       <c r="K58" s="50" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A59" s="40" t="s">
+        <v>180</v>
+      </c>
+      <c r="B59" s="42" t="s">
         <v>181</v>
       </c>
-      <c r="B59" s="42" t="s">
+      <c r="C59" s="42" t="s">
         <v>182</v>
       </c>
-      <c r="C59" s="42" t="s">
+      <c r="D59" s="40" t="s">
         <v>183</v>
-      </c>
-      <c r="D59" s="40" t="s">
-        <v>184</v>
       </c>
       <c r="E59" s="40">
         <v>3</v>
@@ -3316,21 +3317,21 @@
       <c r="I59" s="40"/>
       <c r="J59" s="40"/>
       <c r="K59" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A60" s="40" t="s">
+        <v>184</v>
+      </c>
+      <c r="B60" s="42" t="s">
         <v>185</v>
       </c>
-      <c r="B60" s="42" t="s">
+      <c r="C60" s="42" t="s">
         <v>186</v>
       </c>
-      <c r="C60" s="42" t="s">
-        <v>187</v>
-      </c>
       <c r="D60" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E60" s="40">
         <v>3</v>
@@ -3345,21 +3346,21 @@
       <c r="I60" s="40"/>
       <c r="J60" s="40"/>
       <c r="K60" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A61" s="40" t="s">
+        <v>187</v>
+      </c>
+      <c r="B61" s="42" t="s">
         <v>188</v>
       </c>
-      <c r="B61" s="42" t="s">
+      <c r="C61" s="42" t="s">
         <v>189</v>
       </c>
-      <c r="C61" s="42" t="s">
-        <v>190</v>
-      </c>
       <c r="D61" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E61" s="40">
         <v>2</v>
@@ -3374,21 +3375,21 @@
       <c r="I61" s="40"/>
       <c r="J61" s="40"/>
       <c r="K61" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" s="39">
         <v>8.6</v>
       </c>
       <c r="B62" s="42" t="s">
+        <v>190</v>
+      </c>
+      <c r="C62" s="42" t="s">
         <v>191</v>
       </c>
-      <c r="C62" s="42" t="s">
-        <v>192</v>
-      </c>
       <c r="D62" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E62" s="40">
         <v>2</v>
@@ -3403,15 +3404,15 @@
       <c r="I62" s="40"/>
       <c r="J62" s="40"/>
       <c r="K62" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" s="35" t="s">
+        <v>192</v>
+      </c>
+      <c r="B63" s="43" t="s">
         <v>193</v>
-      </c>
-      <c r="B63" s="43" t="s">
-        <v>194</v>
       </c>
       <c r="C63" s="43"/>
       <c r="D63" s="35"/>
@@ -3422,21 +3423,21 @@
       <c r="I63" s="35"/>
       <c r="J63" s="35"/>
       <c r="K63" s="51" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" s="40" t="s">
+        <v>194</v>
+      </c>
+      <c r="B64" s="42" t="s">
         <v>195</v>
       </c>
-      <c r="B64" s="42" t="s">
+      <c r="C64" s="42" t="s">
         <v>196</v>
       </c>
-      <c r="C64" s="42" t="s">
-        <v>197</v>
-      </c>
       <c r="D64" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E64" s="40">
         <v>1</v>
@@ -3451,21 +3452,21 @@
       <c r="I64" s="40"/>
       <c r="J64" s="40"/>
       <c r="K64" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" s="40" t="s">
+        <v>197</v>
+      </c>
+      <c r="B65" s="42" t="s">
         <v>198</v>
       </c>
-      <c r="B65" s="42" t="s">
+      <c r="C65" s="42" t="s">
         <v>199</v>
       </c>
-      <c r="C65" s="42" t="s">
-        <v>200</v>
-      </c>
       <c r="D65" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E65" s="40">
         <v>1</v>
@@ -3480,21 +3481,21 @@
       <c r="I65" s="40"/>
       <c r="J65" s="40"/>
       <c r="K65" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A66" s="40" t="s">
+        <v>200</v>
+      </c>
+      <c r="B66" s="42" t="s">
         <v>201</v>
       </c>
-      <c r="B66" s="42" t="s">
+      <c r="C66" s="42" t="s">
         <v>202</v>
       </c>
-      <c r="C66" s="42" t="s">
-        <v>203</v>
-      </c>
       <c r="D66" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E66" s="40">
         <v>1</v>
@@ -3509,15 +3510,15 @@
       <c r="I66" s="40"/>
       <c r="J66" s="40"/>
       <c r="K66" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" s="35" t="s">
+        <v>203</v>
+      </c>
+      <c r="B67" s="43" t="s">
         <v>204</v>
-      </c>
-      <c r="B67" s="43" t="s">
-        <v>205</v>
       </c>
       <c r="C67" s="43"/>
       <c r="D67" s="35"/>
@@ -3528,21 +3529,21 @@
       <c r="I67" s="35"/>
       <c r="J67" s="35"/>
       <c r="K67" s="51" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A68" s="40" t="s">
+        <v>205</v>
+      </c>
+      <c r="B68" s="42" t="s">
         <v>206</v>
       </c>
-      <c r="B68" s="42" t="s">
+      <c r="C68" s="42" t="s">
         <v>207</v>
       </c>
-      <c r="C68" s="42" t="s">
-        <v>208</v>
-      </c>
       <c r="D68" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E68" s="40">
         <v>2</v>
@@ -3561,21 +3562,21 @@
         <v>46203</v>
       </c>
       <c r="K68" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A69" s="40" t="s">
+        <v>208</v>
+      </c>
+      <c r="B69" s="42" t="s">
         <v>209</v>
       </c>
-      <c r="B69" s="42" t="s">
+      <c r="C69" s="42" t="s">
         <v>210</v>
       </c>
-      <c r="C69" s="42" t="s">
-        <v>211</v>
-      </c>
       <c r="D69" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E69" s="40">
         <v>1</v>
@@ -3590,21 +3591,21 @@
       <c r="I69" s="40"/>
       <c r="J69" s="40"/>
       <c r="K69" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" s="40" t="s">
+        <v>211</v>
+      </c>
+      <c r="B70" s="42" t="s">
         <v>212</v>
       </c>
-      <c r="B70" s="42" t="s">
+      <c r="C70" s="42" t="s">
         <v>213</v>
       </c>
-      <c r="C70" s="42" t="s">
-        <v>214</v>
-      </c>
       <c r="D70" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E70" s="40">
         <v>2</v>
@@ -3623,21 +3624,21 @@
         <v>46204</v>
       </c>
       <c r="K70" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" s="40" t="s">
+        <v>214</v>
+      </c>
+      <c r="B71" s="42" t="s">
         <v>215</v>
       </c>
-      <c r="B71" s="42" t="s">
+      <c r="C71" s="42" t="s">
         <v>216</v>
       </c>
-      <c r="C71" s="42" t="s">
-        <v>217</v>
-      </c>
       <c r="D71" s="40" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E71" s="40">
         <v>2</v>
@@ -3656,15 +3657,15 @@
         <v>46204</v>
       </c>
       <c r="K71" s="47" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" s="35" t="s">
+        <v>217</v>
+      </c>
+      <c r="B72" s="43" t="s">
         <v>218</v>
-      </c>
-      <c r="B72" s="43" t="s">
-        <v>219</v>
       </c>
       <c r="C72" s="43"/>
       <c r="D72" s="35"/>
@@ -3675,21 +3676,21 @@
       <c r="I72" s="35"/>
       <c r="J72" s="35"/>
       <c r="K72" s="51" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="40" t="s">
+        <v>219</v>
+      </c>
+      <c r="B73" s="42" t="s">
         <v>220</v>
       </c>
-      <c r="B73" s="42" t="s">
+      <c r="C73" s="42" t="s">
         <v>221</v>
       </c>
-      <c r="C73" s="42" t="s">
-        <v>222</v>
-      </c>
       <c r="D73" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E73" s="40">
         <v>3</v>
@@ -3704,21 +3705,21 @@
       <c r="I73" s="40"/>
       <c r="J73" s="40"/>
       <c r="K73" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A74" s="40" t="s">
+        <v>222</v>
+      </c>
+      <c r="B74" s="42" t="s">
         <v>223</v>
       </c>
-      <c r="B74" s="42" t="s">
+      <c r="C74" s="42" t="s">
         <v>224</v>
       </c>
-      <c r="C74" s="42" t="s">
-        <v>225</v>
-      </c>
       <c r="D74" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E74" s="40">
         <v>2</v>
@@ -3733,21 +3734,21 @@
       <c r="I74" s="40"/>
       <c r="J74" s="40"/>
       <c r="K74" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="40" t="s">
+        <v>225</v>
+      </c>
+      <c r="B75" s="42" t="s">
         <v>226</v>
       </c>
-      <c r="B75" s="42" t="s">
+      <c r="C75" s="42" t="s">
         <v>227</v>
       </c>
-      <c r="C75" s="42" t="s">
-        <v>228</v>
-      </c>
       <c r="D75" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E75" s="40">
         <v>2</v>
@@ -3762,21 +3763,21 @@
       <c r="I75" s="40"/>
       <c r="J75" s="40"/>
       <c r="K75" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A76" s="40" t="s">
+        <v>228</v>
+      </c>
+      <c r="B76" s="42" t="s">
         <v>229</v>
       </c>
-      <c r="B76" s="42" t="s">
+      <c r="C76" s="42" t="s">
         <v>230</v>
       </c>
-      <c r="C76" s="42" t="s">
-        <v>231</v>
-      </c>
       <c r="D76" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E76" s="40">
         <v>2</v>
@@ -3791,15 +3792,15 @@
       <c r="I76" s="40"/>
       <c r="J76" s="40"/>
       <c r="K76" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" s="35" t="s">
+        <v>231</v>
+      </c>
+      <c r="B77" s="43" t="s">
         <v>232</v>
-      </c>
-      <c r="B77" s="43" t="s">
-        <v>233</v>
       </c>
       <c r="C77" s="43"/>
       <c r="D77" s="35"/>
@@ -3810,21 +3811,21 @@
       <c r="I77" s="35"/>
       <c r="J77" s="35"/>
       <c r="K77" s="51" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A78" s="40" t="s">
+        <v>233</v>
+      </c>
+      <c r="B78" s="42" t="s">
         <v>234</v>
       </c>
-      <c r="B78" s="42" t="s">
+      <c r="C78" s="42" t="s">
         <v>235</v>
       </c>
-      <c r="C78" s="42" t="s">
-        <v>236</v>
-      </c>
       <c r="D78" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E78" s="40">
         <v>3</v>
@@ -3839,21 +3840,21 @@
       <c r="I78" s="40"/>
       <c r="J78" s="40"/>
       <c r="K78" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A79" s="40" t="s">
+        <v>236</v>
+      </c>
+      <c r="B79" s="42" t="s">
         <v>237</v>
       </c>
-      <c r="B79" s="42" t="s">
+      <c r="C79" s="42" t="s">
         <v>238</v>
       </c>
-      <c r="C79" s="42" t="s">
-        <v>239</v>
-      </c>
       <c r="D79" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E79" s="40">
         <v>3</v>
@@ -3868,21 +3869,21 @@
       <c r="I79" s="40"/>
       <c r="J79" s="40"/>
       <c r="K79" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A80" s="40" t="s">
+        <v>239</v>
+      </c>
+      <c r="B80" s="42" t="s">
         <v>240</v>
       </c>
-      <c r="B80" s="42" t="s">
+      <c r="C80" s="42" t="s">
         <v>241</v>
       </c>
-      <c r="C80" s="42" t="s">
-        <v>242</v>
-      </c>
       <c r="D80" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E80" s="40">
         <v>3</v>
@@ -3897,15 +3898,15 @@
       <c r="I80" s="40"/>
       <c r="J80" s="40"/>
       <c r="K80" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" s="35" t="s">
+        <v>242</v>
+      </c>
+      <c r="B81" s="43" t="s">
         <v>243</v>
-      </c>
-      <c r="B81" s="43" t="s">
-        <v>244</v>
       </c>
       <c r="C81" s="43"/>
       <c r="D81" s="35"/>
@@ -3916,21 +3917,21 @@
       <c r="I81" s="35"/>
       <c r="J81" s="35"/>
       <c r="K81" s="51" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A82" s="40" t="s">
+        <v>244</v>
+      </c>
+      <c r="B82" s="42" t="s">
         <v>245</v>
       </c>
-      <c r="B82" s="42" t="s">
+      <c r="C82" s="42" t="s">
         <v>246</v>
       </c>
-      <c r="C82" s="42" t="s">
-        <v>247</v>
-      </c>
       <c r="D82" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E82" s="40">
         <v>3</v>
@@ -3945,21 +3946,21 @@
       <c r="I82" s="40"/>
       <c r="J82" s="40"/>
       <c r="K82" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" s="40" t="s">
+        <v>247</v>
+      </c>
+      <c r="B83" s="42" t="s">
         <v>248</v>
       </c>
-      <c r="B83" s="42" t="s">
+      <c r="C83" s="42" t="s">
         <v>249</v>
       </c>
-      <c r="C83" s="42" t="s">
-        <v>250</v>
-      </c>
       <c r="D83" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E83" s="40">
         <v>2</v>
@@ -3974,21 +3975,21 @@
       <c r="I83" s="40"/>
       <c r="J83" s="40"/>
       <c r="K83" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" s="40" t="s">
+        <v>250</v>
+      </c>
+      <c r="B84" s="42" t="s">
         <v>251</v>
       </c>
-      <c r="B84" s="42" t="s">
+      <c r="C84" s="42" t="s">
         <v>252</v>
       </c>
-      <c r="C84" s="42" t="s">
-        <v>253</v>
-      </c>
       <c r="D84" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E84" s="40">
         <v>2</v>
@@ -4003,15 +4004,15 @@
       <c r="I84" s="40"/>
       <c r="J84" s="40"/>
       <c r="K84" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" s="35" t="s">
+        <v>253</v>
+      </c>
+      <c r="B85" s="43" t="s">
         <v>254</v>
-      </c>
-      <c r="B85" s="43" t="s">
-        <v>255</v>
       </c>
       <c r="C85" s="43"/>
       <c r="D85" s="35"/>
@@ -4022,21 +4023,21 @@
       <c r="I85" s="35"/>
       <c r="J85" s="35"/>
       <c r="K85" s="51" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" ht="27" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" ht="26.25" x14ac:dyDescent="0.25">
       <c r="A86" s="40" t="s">
+        <v>255</v>
+      </c>
+      <c r="B86" s="42" t="s">
         <v>256</v>
       </c>
-      <c r="B86" s="42" t="s">
+      <c r="C86" s="42" t="s">
         <v>257</v>
       </c>
-      <c r="C86" s="42" t="s">
-        <v>258</v>
-      </c>
       <c r="D86" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E86" s="40">
         <v>1</v>
@@ -4051,21 +4052,21 @@
       <c r="I86" s="40"/>
       <c r="J86" s="40"/>
       <c r="K86" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" s="40" t="s">
+        <v>258</v>
+      </c>
+      <c r="B87" s="42" t="s">
         <v>259</v>
       </c>
-      <c r="B87" s="42" t="s">
+      <c r="C87" s="42" t="s">
         <v>260</v>
       </c>
-      <c r="C87" s="42" t="s">
-        <v>261</v>
-      </c>
       <c r="D87" s="40" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E87" s="40">
         <v>1</v>
@@ -4080,27 +4081,27 @@
       <c r="I87" s="40"/>
       <c r="J87" s="40"/>
       <c r="K87" s="47" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" ht="28.2" x14ac:dyDescent="0.3">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="A88" s="37" t="s">
+        <v>261</v>
+      </c>
+      <c r="B88" s="44" t="s">
         <v>262</v>
       </c>
-      <c r="B88" s="44" t="s">
-        <v>263</v>
-      </c>
       <c r="C88" s="44" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D88" s="37" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E88" s="37">
         <v>0</v>
       </c>
       <c r="F88" s="37" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G88" s="38">
         <v>46224</v>
@@ -4111,7 +4112,7 @@
       <c r="I88" s="37"/>
       <c r="J88" s="37"/>
       <c r="K88" s="52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
@@ -4123,110 +4124,110 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B19"/>
-  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
         <v>264</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="B3" s="4" t="s">
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
         <v>266</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>267</v>
       </c>
-      <c r="B4" s="4" t="s">
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>268</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>269</v>
       </c>
-      <c r="B5" s="4" t="s">
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="7" t="s">
+      <c r="B6" s="4" t="s">
         <v>271</v>
       </c>
-      <c r="B6" s="4" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="8"/>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A7" s="8"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A8" s="8" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" s="9" t="s">
         <v>273</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A10" s="9" t="s">
         <v>274</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A10" s="9" t="s">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
         <v>275</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" s="9" t="s">
         <v>276</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A12" s="9" t="s">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" s="9" t="s">
         <v>277</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
         <v>278</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A15" s="9" t="s">
         <v>279</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A15" s="9" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A16" s="9" t="s">
         <v>280</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="9" t="s">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="9" t="s">
         <v>281</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A17" s="9" t="s">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="9" t="s">
         <v>282</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A18" s="9" t="s">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="9" t="s">
         <v>283</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A19" s="9" t="s">
-        <v>284</v>
       </c>
     </row>
   </sheetData>

</xml_diff>